<commit_message>
Convert SWI-PRO-MET-205-001, 002, 006, 012, 013, 015, 017 to Heritage per Martabe decisions; all series complete
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UHnSDEBA56GANs2gfXuK2P
</commit_message>
<xml_diff>
--- a/docs/Register-SWI-205.xlsx
+++ b/docs/Register-SWI-205.xlsx
@@ -12,8 +12,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Keterangan" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Register 205'!$A$1:$Q$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Draft dan open items'!$A$1:$D$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Register 205'!$A$1:$Q$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Draft dan open items'!$A$1:$D$12</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -35,7 +35,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -45,6 +45,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F3864"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8CBAD"/>
       </patternFill>
     </fill>
     <fill>
@@ -79,7 +89,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -90,7 +100,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -461,7 +477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q13"/>
+  <dimension ref="A1:Q20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -573,17 +589,17 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>205-003</t>
+          <t>205-001</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>SWI-PRO-MET-205-003</t>
+          <t>SWI-PRO-MET-205-001</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>Sulphuric Acid Strength Titration</t>
+          <t>Free Cyanide Titration - Silver Nitrate Method</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
@@ -598,7 +614,7 @@
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>JSEA-PRO-MET-205-003</t>
+          <t>JSEA-PRO-MET-205-001</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -623,18 +639,18 @@
       </c>
       <c r="K2" s="3" t="inlineStr">
         <is>
-          <t>Every made-up batch and once per shift on standing solution.</t>
+          <t>Every shift on every cyanide-bearing stream on the schedule.</t>
         </is>
       </c>
       <c r="L2" s="2" t="n">
         <v>5</v>
       </c>
       <c r="M2" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N2" s="3" t="inlineStr">
         <is>
-          <t>Tidak ada padanan</t>
+          <t>Cyanide Measurement by AgNO3 Titration - pembanding; diambil cek buret digital 0.00 dan kedaluwarsa AgNO3</t>
         </is>
       </c>
       <c r="O2" s="3" t="inlineStr">
@@ -649,24 +665,24 @@
       </c>
       <c r="Q2" s="3" t="inlineStr">
         <is>
-          <t>MM-4034-033-OR-03-SWI-PRO-MET-205-003-Sulphuric-Acid-Strength-Titration-RevA.docx</t>
+          <t>MM-4034-033-OR-03-SWI-PRO-MET-205-001-Free-Cyanide-Titration---Silver-Nitrate-Method-RevA.docx</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>205-004</t>
+          <t>205-002</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>SWI-PRO-MET-205-004</t>
+          <t>SWI-PRO-MET-205-002</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Sodium Chloride (Chloride) Titration</t>
+          <t>Caustic Soda Strength Titration</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
@@ -681,7 +697,7 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>JSEA-PRO-MET-205-004</t>
+          <t>JSEA-PRO-MET-205-002</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -706,23 +722,23 @@
       </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>Every made-up batch and per the analysis schedule.</t>
+          <t>Every made-up batch and once per shift on standing solution.</t>
         </is>
       </c>
       <c r="L3" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M3" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N3" s="3" t="inlineStr">
         <is>
-          <t>Tidak ada padanan</t>
-        </is>
-      </c>
-      <c r="O3" s="3" t="inlineStr">
-        <is>
-          <t>Final (isi tanpa tambahan)</t>
+          <t>ReCYN Plant Caustic Strength Measurement dan Sodium Hydroxide Titration - Step 4 (titrasi H2SO4 alternatif)</t>
+        </is>
+      </c>
+      <c r="O3" s="4" t="inlineStr">
+        <is>
+          <t>DRAFT FOR REVIEW (tambahan Martabe)</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
@@ -732,24 +748,24 @@
       </c>
       <c r="Q3" s="3" t="inlineStr">
         <is>
-          <t>MM-4034-033-OR-03-SWI-PRO-MET-205-004-Sodium-Chloride-Chloride-Titration-RevA.docx</t>
+          <t>MM-4034-033-OR-03-SWI-PRO-MET-205-002-Caustic-Soda-Strength-Titration-RevA.docx</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>205-005</t>
+          <t>205-003</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>SWI-PRO-MET-205-005</t>
+          <t>SWI-PRO-MET-205-003</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Lime Availability Test</t>
+          <t>Sulphuric Acid Strength Titration</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -759,12 +775,12 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Operating</t>
+          <t>Safety-critical</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>JSEA-PRO-MET-205-005</t>
+          <t>JSEA-PRO-MET-205-003</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -789,7 +805,7 @@
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>Every delivery and weekly on the slaked slurry.</t>
+          <t>Every made-up batch and once per shift on standing solution.</t>
         </is>
       </c>
       <c r="L4" s="2" t="n">
@@ -815,24 +831,24 @@
       </c>
       <c r="Q4" s="3" t="inlineStr">
         <is>
-          <t>MM-4034-033-OR-03-SWI-PRO-MET-205-005-Lime-Availability-Test-RevA.docx</t>
+          <t>MM-4034-033-OR-03-SWI-PRO-MET-205-003-Sulphuric-Acid-Strength-Titration-RevA.docx</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>205-007</t>
+          <t>205-004</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>SWI-PRO-MET-205-007</t>
+          <t>SWI-PRO-MET-205-004</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Bottle Roll Leach Test - As-Received and Pulverised</t>
+          <t>Sodium Chloride (Chloride) Titration</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -842,12 +858,12 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>Safety-critical</t>
+          <t>Operating</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>JSEA-PRO-MET-205-007</t>
+          <t>JSEA-PRO-MET-205-004</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -872,14 +888,14 @@
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>On each new ore type, and on any tail sample being investigated.</t>
+          <t>Every made-up batch and per the analysis schedule.</t>
         </is>
       </c>
       <c r="L5" s="2" t="n">
         <v>5</v>
       </c>
       <c r="M5" s="2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="N5" s="3" t="inlineStr">
         <is>
@@ -898,24 +914,24 @@
       </c>
       <c r="Q5" s="3" t="inlineStr">
         <is>
-          <t>MM-4034-033-OR-03-SWI-PRO-MET-205-007-Bottle-Roll-Leach-Test---As-Received-and-Pulverised-RevA.docx</t>
+          <t>MM-4034-033-OR-03-SWI-PRO-MET-205-004-Sodium-Chloride-Chloride-Titration-RevA.docx</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>205-008</t>
+          <t>205-005</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>SWI-PRO-MET-205-008</t>
+          <t>SWI-PRO-MET-205-005</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Extended and Diagnostic Leach Test</t>
+          <t>Lime Availability Test</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
@@ -925,12 +941,12 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>Safety-critical</t>
+          <t>Operating</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>JSEA-PRO-MET-205-008</t>
+          <t>JSEA-PRO-MET-205-005</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -955,14 +971,14 @@
       </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
-          <t>On tail investigation and on each new ore type.</t>
+          <t>Every delivery and weekly on the slaked slurry.</t>
         </is>
       </c>
       <c r="L6" s="2" t="n">
         <v>5</v>
       </c>
       <c r="M6" s="2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="N6" s="3" t="inlineStr">
         <is>
@@ -981,24 +997,24 @@
       </c>
       <c r="Q6" s="3" t="inlineStr">
         <is>
-          <t>MM-4034-033-OR-03-SWI-PRO-MET-205-008-Extended-and-Diagnostic-Leach-Test-RevA.docx</t>
+          <t>MM-4034-033-OR-03-SWI-PRO-MET-205-005-Lime-Availability-Test-RevA.docx</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>205-009</t>
+          <t>205-006</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>SWI-PRO-MET-205-009</t>
+          <t>SWI-PRO-MET-205-006</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>CIL/CIP Sequential Triple Contact Testwork</t>
+          <t>Lime Addition and Lime Demand Test</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
@@ -1008,12 +1024,12 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>Safety-critical</t>
+          <t>Operating</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>JSEA-PRO-MET-205-009</t>
+          <t>JSEA-PRO-MET-205-006</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -1038,23 +1054,23 @@
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>On each new ore type and when adsorption performance is being investigated.</t>
+          <t>On each new ore type and whenever plant lime consumption moves; neutralisation tests when the metallurgist requests them.</t>
         </is>
       </c>
       <c r="L7" s="2" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="M7" s="2" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="N7" s="3" t="inlineStr">
         <is>
-          <t>Tidak ada padanan</t>
-        </is>
-      </c>
-      <c r="O7" s="3" t="inlineStr">
-        <is>
-          <t>Final (isi tanpa tambahan)</t>
+          <t>Dosing NaOH vs Ca(OH)2, MHR1 quicklime (udara, H2O2), MHR1 quicklime dan caustic, TSF Toe (dari 205-015) - digabung jadi Step 4-7, sampel bebas sianida</t>
+        </is>
+      </c>
+      <c r="O7" s="4" t="inlineStr">
+        <is>
+          <t>DRAFT FOR REVIEW (tambahan Martabe)</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
@@ -1064,24 +1080,24 @@
       </c>
       <c r="Q7" s="3" t="inlineStr">
         <is>
-          <t>MM-4034-033-OR-03-SWI-PRO-MET-205-009-CILCIP-Sequential-Triple-Contact-Testwork-RevA.docx</t>
+          <t>MM-4034-033-OR-03-SWI-PRO-MET-205-006-Lime-Addition-and-Lime-Demand-Test-RevA.docx</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>205-010</t>
+          <t>205-007</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>SWI-PRO-MET-205-010</t>
+          <t>SWI-PRO-MET-205-007</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Carbon Adsorption Capacity and Isotherm Test</t>
+          <t>Bottle Roll Leach Test - As-Received and Pulverised</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
@@ -1091,12 +1107,12 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>Operating</t>
+          <t>Safety-critical</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>JSEA-PRO-MET-205-010</t>
+          <t>JSEA-PRO-MET-205-007</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -1121,14 +1137,14 @@
       </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
-          <t>Monthly, and on every new carbon delivery.</t>
+          <t>On each new ore type, and on any tail sample being investigated.</t>
         </is>
       </c>
       <c r="L8" s="2" t="n">
         <v>5</v>
       </c>
       <c r="M8" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N8" s="3" t="inlineStr">
         <is>
@@ -1147,24 +1163,24 @@
       </c>
       <c r="Q8" s="3" t="inlineStr">
         <is>
-          <t>MM-4034-033-OR-03-SWI-PRO-MET-205-010-Carbon-Adsorption-Capacity-and-Isotherm-Test-RevA.docx</t>
+          <t>MM-4034-033-OR-03-SWI-PRO-MET-205-007-Bottle-Roll-Leach-Test---As-Received-and-Pulverised-RevA.docx</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>205-011</t>
+          <t>205-008</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>SWI-PRO-MET-205-011</t>
+          <t>SWI-PRO-MET-205-008</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Carbon Activity and Ball-Pan Hardness Test</t>
+          <t>Extended and Diagnostic Leach Test</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
@@ -1174,12 +1190,12 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>Operating</t>
+          <t>Safety-critical</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>JSEA-PRO-MET-205-011</t>
+          <t>JSEA-PRO-MET-205-008</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -1204,14 +1220,14 @@
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
-          <t>Monthly, and on every new carbon delivery.</t>
+          <t>On tail investigation and on each new ore type.</t>
         </is>
       </c>
       <c r="L9" s="2" t="n">
         <v>5</v>
       </c>
       <c r="M9" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N9" s="3" t="inlineStr">
         <is>
@@ -1230,24 +1246,24 @@
       </c>
       <c r="Q9" s="3" t="inlineStr">
         <is>
-          <t>MM-4034-033-OR-03-SWI-PRO-MET-205-011-Carbon-Activity-and-Ball-Pan-Hardness-Test-RevA.docx</t>
+          <t>MM-4034-033-OR-03-SWI-PRO-MET-205-008-Extended-and-Diagnostic-Leach-Test-RevA.docx</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>205-014</t>
+          <t>205-009</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>SWI-PRO-MET-205-014</t>
+          <t>SWI-PRO-MET-205-009</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Resin Fouling, Osmotic Shock and Bead Integrity Assessment</t>
+          <t>CIL/CIP Sequential Triple Contact Testwork</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
@@ -1257,12 +1273,12 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>Operating</t>
+          <t>Safety-critical</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>JSEA-PRO-MET-205-014</t>
+          <t>JSEA-PRO-MET-205-009</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -1287,7 +1303,7 @@
       </c>
       <c r="K10" s="3" t="inlineStr">
         <is>
-          <t>Monthly, and after any osmotic shock event.</t>
+          <t>On each new ore type and when adsorption performance is being investigated.</t>
         </is>
       </c>
       <c r="L10" s="2" t="n">
@@ -1313,24 +1329,24 @@
       </c>
       <c r="Q10" s="3" t="inlineStr">
         <is>
-          <t>MM-4034-033-OR-03-SWI-PRO-MET-205-014-Resin-Fouling-Osmotic-Shock-and-Bead-Integrity-Assessment-RevA.docx</t>
+          <t>MM-4034-033-OR-03-SWI-PRO-MET-205-009-CILCIP-Sequential-Triple-Contact-Testwork-RevA.docx</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>205-016</t>
+          <t>205-010</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>SWI-PRO-MET-205-016</t>
+          <t>SWI-PRO-MET-205-010</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Precipitate and Platelet Content Determination</t>
+          <t>Carbon Adsorption Capacity and Isotherm Test</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
@@ -1345,7 +1361,7 @@
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>JSEA-PRO-MET-205-016</t>
+          <t>JSEA-PRO-MET-205-010</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -1370,7 +1386,7 @@
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
-          <t>Every lot and per the analysis schedule.</t>
+          <t>Monthly, and on every new carbon delivery.</t>
         </is>
       </c>
       <c r="L11" s="2" t="n">
@@ -1396,24 +1412,24 @@
       </c>
       <c r="Q11" s="3" t="inlineStr">
         <is>
-          <t>MM-4034-033-OR-03-SWI-PRO-MET-205-016-Precipitate-and-Platelet-Content-Determination-RevA.docx</t>
+          <t>MM-4034-033-OR-03-SWI-PRO-MET-205-010-Carbon-Adsorption-Capacity-and-Isotherm-Test-RevA.docx</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>205-018</t>
+          <t>205-011</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>SWI-PRO-MET-205-018</t>
+          <t>SWI-PRO-MET-205-011</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Automatic Titrator Operation and Method Set-Up</t>
+          <t>Carbon Activity and Ball-Pan Hardness Test</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
@@ -1428,7 +1444,7 @@
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>JSEA-PRO-MET-205-018</t>
+          <t>JSEA-PRO-MET-205-011</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -1453,7 +1469,7 @@
       </c>
       <c r="K12" s="3" t="inlineStr">
         <is>
-          <t>At set-up, and whenever a method is added or changed.</t>
+          <t>Monthly, and on every new carbon delivery.</t>
         </is>
       </c>
       <c r="L12" s="2" t="n">
@@ -1479,95 +1495,676 @@
       </c>
       <c r="Q12" s="3" t="inlineStr">
         <is>
-          <t>MM-4034-033-OR-03-SWI-PRO-MET-205-018-Automatic-Titrator-Operation-and-Method-Set-Up-RevA.docx</t>
+          <t>MM-4034-033-OR-03-SWI-PRO-MET-205-011-Carbon-Activity-and-Ball-Pan-Hardness-Test-RevA.docx</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
+          <t>205-012</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>SWI-PRO-MET-205-012</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Resin Adsorption Capacity and Kinetics Test</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>205 Met Lab - Chemical and Leach Testwork</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>Operating</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>JSEA-PRO-MET-205-012</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>11/08/2026</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>11/08/2027</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>Processing</t>
+        </is>
+      </c>
+      <c r="K13" s="3" t="inlineStr">
+        <is>
+          <t>To be set once the vendor data arrives.</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="M13" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="N13" s="3" t="inlineStr">
+        <is>
+          <t>Resin Activity Test dan Adsorption Test Fresh Resin - Step 2-6; varian KCN tidak dipakai; CIL 7 dipetakan ke 032-TK-006</t>
+        </is>
+      </c>
+      <c r="O13" s="4" t="inlineStr">
+        <is>
+          <t>DRAFT FOR REVIEW (tambahan Martabe)</t>
+        </is>
+      </c>
+      <c r="P13" s="2" t="inlineStr">
+        <is>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="Q13" s="3" t="inlineStr">
+        <is>
+          <t>MM-4034-033-OR-03-SWI-PRO-MET-205-012-Resin-Adsorption-Capacity-and-Kinetics-Test-RevA.docx</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>205-013</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>SWI-PRO-MET-205-013</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>Resin Elution Efficiency and Barren Resin Loading Test</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>205 Met Lab - Chemical and Leach Testwork</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>Operating</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>JSEA-PRO-MET-205-013</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>11/08/2026</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>11/08/2027</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>Processing</t>
+        </is>
+      </c>
+      <c r="K14" s="3" t="inlineStr">
+        <is>
+          <t>To be set once the vendor data arrives.</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="M14" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="N14" s="3" t="inlineStr">
+        <is>
+          <t>NaCl vendor, Preconditioning V2, Sulfamic acid, IPHK, Copper Loading Test, Grundfos DDA - Step 2-10</t>
+        </is>
+      </c>
+      <c r="O14" s="4" t="inlineStr">
+        <is>
+          <t>DRAFT FOR REVIEW (tambahan Martabe)</t>
+        </is>
+      </c>
+      <c r="P14" s="2" t="inlineStr">
+        <is>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="Q14" s="3" t="inlineStr">
+        <is>
+          <t>MM-4034-033-OR-03-SWI-PRO-MET-205-013-Resin-Elution-Efficiency-and-Barren-Resin-Loading-Test-RevA.docx</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>205-014</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>SWI-PRO-MET-205-014</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Resin Fouling, Osmotic Shock and Bead Integrity Assessment</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>205 Met Lab - Chemical and Leach Testwork</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>Operating</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>JSEA-PRO-MET-205-014</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>11/08/2026</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>11/08/2027</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>Processing</t>
+        </is>
+      </c>
+      <c r="K15" s="3" t="inlineStr">
+        <is>
+          <t>Monthly, and after any osmotic shock event.</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="M15" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="N15" s="3" t="inlineStr">
+        <is>
+          <t>Tidak ada padanan</t>
+        </is>
+      </c>
+      <c r="O15" s="3" t="inlineStr">
+        <is>
+          <t>Final (isi tanpa tambahan)</t>
+        </is>
+      </c>
+      <c r="P15" s="2" t="inlineStr">
+        <is>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="Q15" s="3" t="inlineStr">
+        <is>
+          <t>MM-4034-033-OR-03-SWI-PRO-MET-205-014-Resin-Fouling-Osmotic-Shock-and-Bead-Integrity-Assessment-RevA.docx</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>205-015</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>SWI-PRO-MET-205-015</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Cyanide Destruction (Detox) Bench Test</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>205 Met Lab - Chemical and Leach Testwork</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>Safety-critical</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>JSEA-PRO-MET-205-015</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>11/08/2026</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>11/08/2027</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>Processing</t>
+        </is>
+      </c>
+      <c r="K16" s="3" t="inlineStr">
+        <is>
+          <t>To be set once the route is chosen.</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="M16" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="N16" s="3" t="inlineStr">
+        <is>
+          <t>TSF Toe to WPP Test - dipindah ke 205-006 (Mt. Morgan tidak punya sirkuit detox)</t>
+        </is>
+      </c>
+      <c r="O16" s="5" t="inlineStr">
+        <is>
+          <t>NOT FOR USE (menunggu input)</t>
+        </is>
+      </c>
+      <c r="P16" s="2" t="inlineStr">
+        <is>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="Q16" s="3" t="inlineStr">
+        <is>
+          <t>MM-4034-033-OR-03-SWI-PRO-MET-205-015-Cyanide-Destruction-Detox-Bench-Test-RevA.docx</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>205-016</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>SWI-PRO-MET-205-016</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Precipitate and Platelet Content Determination</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>205 Met Lab - Chemical and Leach Testwork</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>Operating</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>JSEA-PRO-MET-205-016</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>11/08/2026</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>11/08/2027</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>Processing</t>
+        </is>
+      </c>
+      <c r="K17" s="3" t="inlineStr">
+        <is>
+          <t>Every lot and per the analysis schedule.</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="M17" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="N17" s="3" t="inlineStr">
+        <is>
+          <t>Tidak ada padanan</t>
+        </is>
+      </c>
+      <c r="O17" s="3" t="inlineStr">
+        <is>
+          <t>Final (isi tanpa tambahan)</t>
+        </is>
+      </c>
+      <c r="P17" s="2" t="inlineStr">
+        <is>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="Q17" s="3" t="inlineStr">
+        <is>
+          <t>MM-4034-033-OR-03-SWI-PRO-MET-205-016-Precipitate-and-Platelet-Content-Determination-RevA.docx</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>205-017</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>SWI-PRO-MET-205-017</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>Preparation of Standard and Working Solutions</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>205 Met Lab - Chemical and Leach Testwork</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>Safety-critical</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>JSEA-PRO-MET-205-017</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>11/08/2026</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>11/08/2027</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>Processing</t>
+        </is>
+      </c>
+      <c r="K18" s="3" t="inlineStr">
+        <is>
+          <t>As the solution register requires; standards re-standardised at the set interval.</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="M18" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="N18" s="3" t="inlineStr">
+        <is>
+          <t>Testwork QC Expired Reagent - Step 5-6, terbatas phenolphthalein dan silica gel</t>
+        </is>
+      </c>
+      <c r="O18" s="4" t="inlineStr">
+        <is>
+          <t>DRAFT FOR REVIEW (tambahan Martabe)</t>
+        </is>
+      </c>
+      <c r="P18" s="2" t="inlineStr">
+        <is>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="Q18" s="3" t="inlineStr">
+        <is>
+          <t>MM-4034-033-OR-03-SWI-PRO-MET-205-017-Preparation-of-Standard-and-Working-Solutions-RevA.docx</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>205-018</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>SWI-PRO-MET-205-018</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Automatic Titrator Operation and Method Set-Up</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>205 Met Lab - Chemical and Leach Testwork</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>Operating</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>JSEA-PRO-MET-205-018</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>11/08/2026</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>11/08/2027</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>Processing</t>
+        </is>
+      </c>
+      <c r="K19" s="3" t="inlineStr">
+        <is>
+          <t>At set-up, and whenever a method is added or changed.</t>
+        </is>
+      </c>
+      <c r="L19" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="M19" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="N19" s="3" t="inlineStr">
+        <is>
+          <t>Tidak ada padanan</t>
+        </is>
+      </c>
+      <c r="O19" s="3" t="inlineStr">
+        <is>
+          <t>Final (isi tanpa tambahan)</t>
+        </is>
+      </c>
+      <c r="P19" s="2" t="inlineStr">
+        <is>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="Q19" s="3" t="inlineStr">
+        <is>
+          <t>MM-4034-033-OR-03-SWI-PRO-MET-205-018-Automatic-Titrator-Operation-and-Method-Set-Up-RevA.docx</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
           <t>205-019</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B20" s="3" t="inlineStr">
         <is>
           <t>SWI-PRO-MET-205-019</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr">
+      <c r="C20" s="3" t="inlineStr">
         <is>
           <t>Automatic Titrator Electrode Care, Standardisation and Verification</t>
         </is>
       </c>
-      <c r="D13" s="3" t="inlineStr">
+      <c r="D20" s="3" t="inlineStr">
         <is>
           <t>205 Met Lab - Chemical and Leach Testwork</t>
         </is>
       </c>
-      <c r="E13" s="3" t="inlineStr">
+      <c r="E20" s="3" t="inlineStr">
         <is>
           <t>Operating</t>
         </is>
       </c>
-      <c r="F13" s="3" t="inlineStr">
+      <c r="F20" s="3" t="inlineStr">
         <is>
           <t>JSEA-PRO-MET-205-019</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="G20" s="2" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="H13" s="2" t="inlineStr">
+      <c r="H20" s="2" t="inlineStr">
         <is>
           <t>11/08/2026</t>
         </is>
       </c>
-      <c r="I13" s="2" t="inlineStr">
+      <c r="I20" s="2" t="inlineStr">
         <is>
           <t>11/08/2027</t>
         </is>
       </c>
-      <c r="J13" s="2" t="inlineStr">
+      <c r="J20" s="2" t="inlineStr">
         <is>
           <t>Processing</t>
         </is>
       </c>
-      <c r="K13" s="3" t="inlineStr">
+      <c r="K20" s="3" t="inlineStr">
         <is>
           <t>Daily standardisation; weekly verification; replacement on failure.</t>
         </is>
       </c>
-      <c r="L13" s="2" t="n">
+      <c r="L20" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="M13" s="2" t="n">
+      <c r="M20" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="N13" s="3" t="inlineStr">
+      <c r="N20" s="3" t="inlineStr">
         <is>
           <t>Tidak ada padanan</t>
         </is>
       </c>
-      <c r="O13" s="3" t="inlineStr">
+      <c r="O20" s="3" t="inlineStr">
         <is>
           <t>Final (isi tanpa tambahan)</t>
         </is>
       </c>
-      <c r="P13" s="2" t="inlineStr">
+      <c r="P20" s="2" t="inlineStr">
         <is>
           <t>Sudah</t>
         </is>
       </c>
-      <c r="Q13" s="3" t="inlineStr">
+      <c r="Q20" s="3" t="inlineStr">
         <is>
           <t>MM-4034-033-OR-03-SWI-PRO-MET-205-019-Automatic-Titrator-Electrode-Care-Standardisation-and-Verification-RevA.docx</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q13"/>
+  <autoFilter ref="A1:Q20"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1578,7 +2175,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1588,51 +2185,271 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>No. dokumen</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="B1" s="6" t="inlineStr">
         <is>
           <t>Judul</t>
         </is>
       </c>
-      <c r="C1" s="4" t="inlineStr">
+      <c r="C1" s="6" t="inlineStr">
         <is>
           <t>Jenis</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="D1" s="6" t="inlineStr">
         <is>
           <t>Isi catatan</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="B2" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C2" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D2" s="5" t="inlineStr">
-        <is>
-          <t>Tidak ada draft, catatan, atau open items di seri ini.</t>
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>SWI-PRO-MET-205-002</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>Caustic Soda Strength Titration</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="inlineStr">
+        <is>
+          <t>Draft for review: Step 4 follows the Martabe work instructions ReCYN Plant Caustic Strength Measurement (DOC-3-MET-PMC-WIN-00088-IE) and Sodium Hydroxide Titration (DOC-3-MET-PMC-WIN-00102-IE), v1.0, 25/12/2024, as an alternative titration with standardised sulphuric acid. HCl titration (Step 3) stays the main method. JSEA-PRO-MET-205-002 must be checked before this instruction is approved.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>SWI-PRO-MET-205-002</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>Caustic Soda Strength Titration</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>Open items</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>Open items: (1) the Martabe instruction for preparing the sulphuric acid titrant has not been received - set the make-up and standardisation of the titrant before Step 4 is used.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>SWI-PRO-MET-205-006</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>Lime Addition and Lime Demand Test</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>Draft for review: Steps 4 to 7 combine the Martabe work instructions Dosing NaOH vs Ca(OH)2 to pH 6, 7, 8 and 9, MHR1 Quick Lime Metal Removed, MHR1 Quick Lime and Caustic (V1 and V1.2) and TSF Toe to WPP Test (moved from SWI-PRO-MET-205-015) into one acid water neutralisation method. The Martabe sample names (SP09, MHR-1, TSF Toe) and the numbers in the Martabe record tables are not used. JSEA-PRO-MET-205-006 must be updated for the added hazards before this instruction is approved.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>SWI-PRO-MET-205-006</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>Lime Addition and Lime Demand Test</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>Open items</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>Open items: (1) name the Mt. Morgan acid water streams this test is run on, and their sample points; (2) set the air flow and the way the air is added; (3) set the hydrogen peroxide strength and the dose per litre of sample; (4) confirm the assay laboratory and analyte suite for each water; (5) the Martabe tables report solid reagent in mL/L - report in g/L or kg/m3.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>SWI-PRO-MET-205-012</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>Resin Adsorption Capacity and Kinetics Test</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>Draft for review - NOT FOR USE until approved. Steps 2 to 6 follow the Martabe work instructions Resin Activity Test (03/03/2025) and Adsorption Test Fresh Resin (09/01/2025). The KCN variant of the activity test is not used. The Martabe CIL tank 7 launder to detox is mapped to the discharge of the last CIL tank (032-TK-006) to ReCYN. JSEA-PRO-MET-205-012 must be updated for the added hazards before this instruction is approved.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>SWI-PRO-MET-205-012</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>Resin Adsorption Capacity and Kinetics Test</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>Open items</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>Open items: (1) acceptance targets for GG1200M and GG1200C need Goldquip resin performance data, not received; (2) loading capacity is not covered by the Martabe method - a capacity method is still needed; (3) confirm the sizing screens (1.18 and 1.4 mm in the source, 0.9 mm in this SWI) against the Goldquip resin specification; (4) the CuSO4 solution strength, and the sample the per cent solids check applies to, are not stated; (5) confirm the values highlighted in the source - 150 mL samples, sample times, filtering and the Cu and Fe assay.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>SWI-PRO-MET-205-013</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>Resin Elution Efficiency and Barren Resin Loading Test</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>Draft for review - NOT FOR USE until approved. Steps 2 to 10 follow the Martabe work instructions Testing NaCl from New Vendor (11/01/2025), Preconditioning Resin with Cu Variance V2 (07/02/2025), Testwork Pelarutan Scaling Eluant Garam Menggunakan Sulfamic Acid (07/10/2025), IPHK Mixing Larutan Campuran NaCN-NaCl (undated), Copper Loading Test (DOC-3-MET-MEL-WIN-00113-IE, 25/01/2025) and Dosing Pump Grundfos DDA Calibration (DOC-3-MET-PMC-WIN-00120-IE, 25/12/2024). Preconditioning follows V2. Every cyanide addition is made at pH 10.5 or above. JSEA-PRO-MET-205-013 must be updated for the added hazards before this instruction is approved.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>SWI-PRO-MET-205-013</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Resin Elution Efficiency and Barren Resin Loading Test</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>Open items</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>Open items: (1) acceptance targets need Goldquip resin elution data, not received; (2) the NaCN to CuSO4 ratio differs between the NaCl vendor method and V2 (about 0.107 against 0.15 g/mL), and the CuSO4 solution strength and hydrate are not stated; (3) confirm the eluant strength of 29.4 g NaCN in 600 mL (about 49 g/L); (4) confirm which NaCl sources the four resin charges represent; (5) confirm the plant NaCl and NaCN solution strengths for the mixing test, and what IPHK stands for; (6) the source adds the KCN solution to the zinc sulphate solution, which is slightly acidic - confirm the order with HSE; adding the zinc sulphate to the alkaline KCN keeps the cyanide alkaline; (7) confirm the Mt. Morgan cyanide-bearing route for the hi-cyanide eluate - the Martabe tailing sump pump is a source name; (8) confirm the dosing pump hose connections against the pump manual; (9) confirm the Mt. Morgan worksheets for the elution, copper loading and pump calibration records - the Martabe G: drive files and forms are source names.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>SWI-PRO-MET-205-015</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Cyanide Destruction (Detox) Bench Test</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>Catatan</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>ISSUED BUT NOT FOR USE. Mt. Morgan has no detox circuit - the ReCYN circuit follows CIL. The back-up detox route decision (OR-07) is open and no cyanide destruction route has been chosen, so this bench test cannot be defined. The Martabe TSF Toe to WPP Test is a water neutralisation test and has been moved to SWI-PRO-MET-205-006.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>SWI-PRO-MET-205-017</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Preparation of Standard and Working Solutions</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>Draft for review: Steps 5 and 6 follow the Martabe work instruction Testwork QC Expired Reagent (28/03/2025). Re-qualification is limited to phenolphthalein indicator and silica gel, never standards, primary reagents or cyanide, and needs the approval of the Metallurgy Superintendent. JSEA-PRO-MET-205-017 must be updated for the added hazards before this instruction is approved.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>SWI-PRO-MET-205-017</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Preparation of Standard and Working Solutions</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>Open items</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>Open items: (1) Metallurgy Superintendent approval of the re-qualification policy; (2) the silica gel drying temperature is not stated - take it from the safety data sheet (typically about 110 to 120 deg C); (3) the Martabe Reagent Lifetime Management System (DOC-IV-MET-CHH-SOP-00039) has not been received.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D2"/>
+  <autoFilter ref="A1:D12"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1650,49 +2467,49 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>Register seri 205 Chemical Testwork (12 dokumen dalam format Heritage).</t>
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>Register seri 205 Chemical Testwork (19 dokumen dalam format Heritage).</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="inlineStr">
+      <c r="A2" s="7" t="inlineStr">
         <is>
           <t>Data dibaca langsung dari Part 1 dan Part 2 tiap dokumen (judul, tanggal, owner, JSEA ID, area, frekuensi).</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="7" t="inlineStr">
         <is>
           <t>Klasifikasi dan padanan Martabe diambil dari docs/Matriks-Rujukan-Martabe.xlsx dan docs/Tabel-SWI-vs-Martabe.xlsx, ditimpa oleh keputusan review bila ada. Format Heritage tidak memuat kolom klasifikasi, jadi klasifikasi hanya ada di register.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="A4" s="7" t="inlineStr">
         <is>
           <t>Jumlah step dan halaman dihitung dari render dokumen (LibreOffice); halaman bisa sedikit berbeda di Microsoft Word.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="inlineStr">
+      <c r="A5" s="7" t="inlineStr">
         <is>
           <t>Status isi: Final = tanpa tambahan Martabe terbuka; DRAFT FOR REVIEW = ada tambahan Martabe yang menunggu JSEA; Catatan = ada catatan yang perlu ditindaklanjuti.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="A6" s="7" t="inlineStr">
         <is>
           <t>Sheet "Draft dan open items" memuat paragraf draft, catatan, temuan safety-critical, dan open items di Description of work.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="inlineStr">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>Referensi register: HM-MMM-WHS-REG-XXX-R00-SWI-SWMS, tab SWI-MET.</t>
         </is>

</xml_diff>